<commit_message>
updated sheet with gap analysis
</commit_message>
<xml_diff>
--- a/canada-strong/_data/canada_strong_content_review.xlsx
+++ b/canada-strong/_data/canada_strong_content_review.xlsx
@@ -5,6 +5,7 @@
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
     <sheet name="Content Review" sheetId="2" r:id="rId2"/>
     <sheet name="Decision Tree" sheetId="3" r:id="rId4"/>
+    <sheet name="Gap Analysis" sheetId="4" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -135,7 +136,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A58"/>
+  <dimension ref="A1:A81"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="100" customWidth="1"/>
@@ -164,7 +165,7 @@
     <row r="5" spans="1:1">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">This workbook has two working tabs plus this one.</t>
+          <t xml:space="preserve">This workbook has three working tabs plus this one.</t>
         </is>
       </c>
     </row>
@@ -448,54 +449,207 @@
       <c r="A50" s="12"/>
     </row>
     <row r="51" spans="1:1">
-      <c r="A51" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Both tabs: set Status to Needs change if flagging something for a fix, or Approved</t>
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAB: Gap Analysis</t>
         </is>
       </c>
     </row>
     <row r="52" spans="1:1">
       <c r="A52" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">once happy with a row. Leave as Open otherwise. Add your name under Reviewer.</t>
+          <t xml:space="preserve">  Compares every program named on two live Canada.ca pages - the workers/employers</t>
         </is>
       </c>
     </row>
     <row r="53" spans="1:1">
-      <c r="A53" s="12"/>
+      <c r="A53" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  tariff-support page and the Canada Strong campaign page - against the CSV that</t>
+        </is>
+      </c>
     </row>
     <row r="54" spans="1:1">
-      <c r="A54" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Source files:</t>
+      <c r="A54" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  drives the wizard, to catch anything the wizard is missing.</t>
         </is>
       </c>
     </row>
     <row r="55" spans="1:1">
       <c r="A55" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  canada-strong/_data/canada_strong_en.yml</t>
+          <t xml:space="preserve">    1. Missing - employer/business side       - on the source page, not in the CSV</t>
         </is>
       </c>
     </row>
     <row r="56" spans="1:1">
       <c r="A56" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  canada-strong/_data/canada_strong_fr.yml</t>
+          <t xml:space="preserve">    2. Missing - new program (not in the CSV) - Build Communities Strong Fund</t>
         </is>
       </c>
     </row>
     <row r="57" spans="1:1">
       <c r="A57" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  canada-strong/_data/tariff_tool_links.csv  (the program list behind the Decision Tree tab)</t>
+          <t xml:space="preserve">    3. Missing - worker-facing supports        - out of scope by design: the wizard</t>
         </is>
       </c>
     </row>
     <row r="58" spans="1:1">
       <c r="A58" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">                                                 only covers the business path, and</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" spans="1:1">
+      <c r="A59" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                                 "I am a worker" on the start page</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" spans="1:1">
+      <c r="A60" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                                 routes straight to that source page</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" spans="1:1">
+      <c r="A61" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                                 instead of building a list</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" spans="1:1">
+      <c r="A62" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    4. Confirmed present                       - already in the wizard; Maps to</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" spans="1:1">
+      <c r="A63" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                                 wizard program names the matching</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" spans="1:1">
+      <c r="A64" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                                 CSV / Decision Tree entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" spans="1:1">
+      <c r="A65" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Set Status per row to Add to wizard, Won't add, or leave Open for a call still</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" spans="1:1">
+      <c r="A66" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  to be made; rows already in the wizard default to Already covered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" spans="1:1">
+      <c r="A67" s="12"/>
+    </row>
+    <row r="68" spans="1:1">
+      <c r="A68" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content Review and Decision Tree tabs: set Status to Needs change if flagging</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" spans="1:1">
+      <c r="A69" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">something for a fix, or Approved once happy with a row. Leave as Open otherwise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" spans="1:1">
+      <c r="A70" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add your name under Reviewer on any tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" spans="1:1">
+      <c r="A71" s="12"/>
+    </row>
+    <row r="72" spans="1:1">
+      <c r="A72" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Source files:</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" spans="1:1">
+      <c r="A73" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  canada-strong/_data/canada_strong_en.yml</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" spans="1:1">
+      <c r="A74" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  canada-strong/_data/canada_strong_fr.yml</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" spans="1:1">
+      <c r="A75" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  canada-strong/_data/tariff_tool_links.csv  (the program list behind the Decision Tree tab)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" spans="1:1">
+      <c r="A76" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">  canada-strong/business-en.html  (the template that assembles the results page)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" spans="1:1">
+      <c r="A77" s="12"/>
+    </row>
+    <row r="78" spans="1:1">
+      <c r="A78" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Compared against, for the Gap Analysis tab (checked 2026-09-03):</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" spans="1:1">
+      <c r="A79" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  https://www.canada.ca/en/department-finance/programs/international-trade-finance-policy/</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" spans="1:1">
+      <c r="A80" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    canadas-response-us-tariffs/support-canadian-workers-employers.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" spans="1:1">
+      <c r="A81" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  https://www.canada.ca/en/campaign/canadastrong.html</t>
         </is>
       </c>
     </row>
@@ -7095,4 +7249,1339 @@
     </dataValidation>
   </dataValidations>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I35"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="38" customWidth="1"/>
+    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="50" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="46" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="9" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Category</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Program / Service</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Organization</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Description (from source page)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Source page</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maps to wizard program</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Status</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reviewer</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comments</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Missing - employer/business side</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Job Bank</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Job Bank (ESDC)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resources to help find, hire and retain the right workers, explore the job market and stay informed about employment standards.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F2" s="2"/>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="H2" s="5"/>
+      <c r="I2" s="2"/>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Missing - employer/business side</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Job Bank - Training Finder</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Job Bank (ESDC)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For employers with a Work-Sharing agreement: training and other resources via Job Bank's Training Finder.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="H3" s="5"/>
+      <c r="I3" s="2"/>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Missing - employer/business side</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Job Bank - Worker Search Tool</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Job Bank (ESDC)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Search an occupation to discover the number of workers looking for a job locally or nationwide.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F4" s="2"/>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="H4" s="5"/>
+      <c r="I4" s="2"/>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Missing - employer/business side</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Expanding your business into new markets</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">International Canada</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New market entry, reducing risk, trade data and inclusive trade.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(distinct from EDC's Market diversification guide, which IS in the wizard)</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="H5" s="5"/>
+      <c r="I5" s="2"/>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Missing - employer/business side</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What importers need to know</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CBSA</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resources for businesses importing goods into Canada.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F6" s="2"/>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="H6" s="5"/>
+      <c r="I6" s="2"/>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Missing - employer/business side</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Supporting Canadian exporters</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trade Commissioner Service (GAC)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Explore available resources to navigate U.S. tariffs.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(distinct page from "Support for Canadian exporters faced with U.S. tariffs", which IS in the wizard as the TCS row)</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="H7" s="5"/>
+      <c r="I7" s="2"/>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2. Missing - new program (not in the CSV at all)</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Build Communities Strong Fund</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(not stated on page)</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Investing in a wide range of infrastructure projects that support economic prosperity through housing, health, transit, and climate adaptation.</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Canada Strong campaign page</t>
+        </is>
+      </c>
+      <c r="F8" s="6"/>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="H8" s="9"/>
+      <c r="I8" s="6"/>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. Missing - worker-facing supports (out of scope by design)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Temporary Employment Insurance (EI) Measures</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ESDC</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Measures that improve access to EI benefits, including waiving the one-week EI waiting period.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F9" s="2"/>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="H9" s="5"/>
+      <c r="I9" s="2"/>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. Missing - worker-facing supports (out of scope by design)</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Job Bank (worker-facing)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Job Bank (ESDC)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Job postings and career opportunities - the leading source for jobs and labour market information.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F10" s="2"/>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="H10" s="5"/>
+      <c r="I10" s="2"/>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. Missing - worker-facing supports (out of scope by design)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Skills for Success</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Government of Canada</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assess your skills and learn about the skills necessary to succeed in today's evolving labour market.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F11" s="2"/>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="H11" s="5"/>
+      <c r="I11" s="2"/>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. Missing - worker-facing supports (out of scope by design)</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Training Finder (worker-facing)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Job Bank (ESDC)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gain in-demand skills from training courses by recognized Canadian institutions.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F12" s="2"/>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="H12" s="5"/>
+      <c r="I12" s="2"/>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. Missing - worker-facing supports (out of scope by design)</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Skills and employment training for Indigenous people</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ESDC</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Develop your skills and access job training through Indigenous service organizations.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F13" s="2"/>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="H13" s="5"/>
+      <c r="I13" s="2"/>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. Missing - worker-facing supports (out of scope by design)</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Canada Student Grants and Loans</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Government of Canada</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Grants and loans available to full-time and part-time post-secondary students.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F14" s="2"/>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="H14" s="5"/>
+      <c r="I14" s="2"/>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. Missing - worker-facing supports (out of scope by design)</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repayment Assistance Plan (RAP)</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Government of Canada</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repayment assistance if you are having trouble paying your student loan.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F15" s="2"/>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="H15" s="5"/>
+      <c r="I15" s="2"/>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. Missing - worker-facing supports (out of scope by design)</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Employment Insurance (EI) and courses or training programs</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ESDC</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Take a course or training program while receiving EI benefits.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F16" s="2"/>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="H16" s="5"/>
+      <c r="I16" s="2"/>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. Missing - worker-facing supports (out of scope by design)</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Canada Apprentice Loan</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Government of Canada</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interest-free loans to help complete an apprenticeship in a designated Red Seal trade.</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F17" s="2"/>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="H17" s="5"/>
+      <c r="I17" s="2"/>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. Missing - worker-facing supports (out of scope by design)</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tax deductions and credits for apprentices</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Government of Canada</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tax deductions and credits for tradespeople, including moving expenses, tuition fees and tool expenses.</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F18" s="2"/>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="H18" s="5"/>
+      <c r="I18" s="2"/>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. Missing - worker-facing supports (out of scope by design)</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EI for apprentices</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ESDC</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Income support during full-time technical training.</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F19" s="2"/>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open</t>
+        </is>
+      </c>
+      <c r="H19" s="5"/>
+      <c r="I19" s="2"/>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Confirmed present - already covered</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Work-Sharing Program</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ESDC</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Measures for employers experiencing a temporary reduction in business.</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Work-Sharing Program (ESDC) - workforce, sector-agnostic</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already covered</t>
+        </is>
+      </c>
+      <c r="H20" s="9"/>
+      <c r="I20" s="6"/>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Confirmed present - already covered</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Student Work Placement Program</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ESDC</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wage subsidies to hire post-secondary students.</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Student Work Placement Program (ESDC) - workforce, sector-agnostic</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already covered</t>
+        </is>
+      </c>
+      <c r="H21" s="9"/>
+      <c r="I21" s="6"/>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Confirmed present - already covered</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Worker Retention Grant</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ESDC</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Income support for EI-eligible employees on reduced hours under an approved Work-Sharing agreement.</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Worker Retention Grant (ESDC) - workforce, sector-agnostic</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already covered</t>
+        </is>
+      </c>
+      <c r="H22" s="9"/>
+      <c r="I22" s="6"/>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Confirmed present - already covered</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regional Tariff Response Initiative</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regional development agencies</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Financial support for small and medium-sized enterprises impacted by tariffs.</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Both pages</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regional Tariff Response Initiative (national hub, liquidity/transformation agnostic) + per-region variants in the regional programs block</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already covered</t>
+        </is>
+      </c>
+      <c r="H23" s="9"/>
+      <c r="I23" s="6"/>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Confirmed present - already covered</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Strategic Response Fund</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ISED</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For innovative projects in sectors affected by the U.S. tariffs.</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Strategic Response Fund (SRF) (ISED) - transformation, sector-agnostic</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already covered</t>
+        </is>
+      </c>
+      <c r="H24" s="9"/>
+      <c r="I24" s="6"/>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Confirmed present - already covered</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Large Enterprise Tariff Loan</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CEEFC</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Loans for large Canadian enterprises affected by current and future tariffs and countermeasures.</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Large Enterprise Tariff Loan (LETL) (CEEFC / CDEV) - liquidity, sector-agnostic</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already covered</t>
+        </is>
+      </c>
+      <c r="H25" s="9"/>
+      <c r="I25" s="6"/>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Confirmed present - already covered</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Supports for business</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ISED</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Loans, grants and tailored programs to help a business expand into new markets.</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Supports for business (hub) (ISED) - always-on hub</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already covered</t>
+        </is>
+      </c>
+      <c r="H26" s="9"/>
+      <c r="I26" s="6"/>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Confirmed present - already covered</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Business Benefits Finder</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ISED</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A tailored list of benefits that may be helpful to your business.</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Business Benefits Finder (ISED) - always-on hub</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already covered</t>
+        </is>
+      </c>
+      <c r="H27" s="9"/>
+      <c r="I27" s="6"/>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Confirmed present - already covered</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Process for requesting remission of tariffs</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Finance Canada</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Request exceptional relief from tariffs imposed as part of Canada's countermeasures.</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Process for requesting remission of tariffs (Finance Canada) - liquidity, sector-agnostic</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already covered</t>
+        </is>
+      </c>
+      <c r="H28" s="9"/>
+      <c r="I28" s="6"/>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Confirmed present - already covered</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Support for the Canadian Steel Sector</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Finance Canada</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trade measures, financial support and more to help the steel sector.</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Support for the Canadian steel sector (Finance Canada) - steel sector hub</t>
+        </is>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already covered</t>
+        </is>
+      </c>
+      <c r="H29" s="9"/>
+      <c r="I29" s="6"/>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Confirmed present - already covered</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Support for forest sector</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Natural Resources Canada</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Liquidity support, assistance to affected workers and industry transformation.</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Support for forest sector employers and workers (hub) (NRCan) - forestry sector hub</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already covered</t>
+        </is>
+      </c>
+      <c r="H30" s="9"/>
+      <c r="I30" s="6"/>
+    </row>
+    <row r="31" spans="1:9">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Confirmed present - already covered</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Duties Relief Program</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CBSA</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qualified businesses can apply to import commercial goods without paying duties.</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Duties Relief Program (CBSA) - liquidity, sector-agnostic</t>
+        </is>
+      </c>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already covered</t>
+        </is>
+      </c>
+      <c r="H31" s="9"/>
+      <c r="I31" s="6"/>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Confirmed present - already covered</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drawback Program</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CBSA</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Removing the domestic duty impact from commercial goods to compete in export markets.</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Duty Drawback Program (CBSA) - liquidity, sector-agnostic</t>
+        </is>
+      </c>
+      <c r="G32" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already covered</t>
+        </is>
+      </c>
+      <c r="H32" s="9"/>
+      <c r="I32" s="6"/>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Confirmed present - already covered</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Support for Canadian exporters faced with U.S. tariffs</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trade Commissioner Service (GAC)</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Help on how to export duty-free to the U.S.</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TCS - US tariffs support for exporters (GAC) - transformation, sector-agnostic</t>
+        </is>
+      </c>
+      <c r="G33" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already covered</t>
+        </is>
+      </c>
+      <c r="H33" s="9"/>
+      <c r="I33" s="6"/>
+    </row>
+    <row r="34" spans="1:9">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Confirmed present - already covered</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Employment Insurance-funded Labour Market Development Agreements (LMDAs)</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ESDC</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Government investments through LMDAs to help workers and employers affected by tariffs access training and employment support.</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workforce Tariff Response - EI-funded LMDAs (ESDC) - workforce, sector-agnostic</t>
+        </is>
+      </c>
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already covered</t>
+        </is>
+      </c>
+      <c r="H34" s="9"/>
+      <c r="I34" s="6"/>
+    </row>
+    <row r="35" spans="1:9">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Confirmed present - already covered</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Services for agri-food exporters (partial match)</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AAFC</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Help for agri-food businesses to export goods - trade shows, in-market expertise and the Canada Brand.</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workers-employers page</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Canada Brand (AAFC) + Trade Commissioner Service (agri-food) (AAFC) - agriculture, transformation block</t>
+        </is>
+      </c>
+      <c r="G35" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Already covered</t>
+        </is>
+      </c>
+      <c r="H35" s="9"/>
+      <c r="I35" s="6"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I35"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G35">
+      <formula1>"Open,Add to wizard,Won't add,Already covered"</formula1>
+    </dataValidation>
+  </dataValidations>
+</worksheet>
 </file>
</xml_diff>